<commit_message>
Disconnect fixes for later
</commit_message>
<xml_diff>
--- a/simple_game_test/combined_metrics_analysis.xlsx
+++ b/simple_game_test/combined_metrics_analysis.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N75"/>
+  <dimension ref="A1:N89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4200,6 +4200,706 @@
         <v>8</v>
       </c>
     </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>286</v>
+      </c>
+      <c r="B76" t="n">
+        <v>87</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>common_belief</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>at-sb</t>
+        </is>
+      </c>
+      <c r="F76" t="n">
+        <v>3.666666666666667</v>
+      </c>
+      <c r="G76" t="n">
+        <v>4</v>
+      </c>
+      <c r="H76" t="n">
+        <v>3.333333333333333</v>
+      </c>
+      <c r="I76" t="n">
+        <v>6</v>
+      </c>
+      <c r="J76" t="n">
+        <v>4</v>
+      </c>
+      <c r="K76" t="n">
+        <v>2</v>
+      </c>
+      <c r="L76" t="n">
+        <v>2</v>
+      </c>
+      <c r="M76" t="n">
+        <v>0</v>
+      </c>
+      <c r="N76" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>286</v>
+      </c>
+      <c r="B77" t="n">
+        <v>87</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>sb</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>common_belief</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>at-sb</t>
+        </is>
+      </c>
+      <c r="F77" t="n">
+        <v>3.666666666666667</v>
+      </c>
+      <c r="G77" t="n">
+        <v>4</v>
+      </c>
+      <c r="H77" t="n">
+        <v>3.666666666666667</v>
+      </c>
+      <c r="I77" t="n">
+        <v>6</v>
+      </c>
+      <c r="J77" t="n">
+        <v>4</v>
+      </c>
+      <c r="K77" t="n">
+        <v>1</v>
+      </c>
+      <c r="L77" t="n">
+        <v>1</v>
+      </c>
+      <c r="M77" t="n">
+        <v>2</v>
+      </c>
+      <c r="N77" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>294</v>
+      </c>
+      <c r="B78" t="n">
+        <v>88</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>joint_belief</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>sb-at</t>
+        </is>
+      </c>
+      <c r="F78" t="n">
+        <v>3.666666666666667</v>
+      </c>
+      <c r="G78" t="n">
+        <v>5</v>
+      </c>
+      <c r="H78" t="n">
+        <v>3</v>
+      </c>
+      <c r="I78" t="n">
+        <v>6</v>
+      </c>
+      <c r="J78" t="n">
+        <v>5</v>
+      </c>
+      <c r="K78" t="n">
+        <v>2</v>
+      </c>
+      <c r="L78" t="n">
+        <v>1</v>
+      </c>
+      <c r="M78" t="n">
+        <v>2</v>
+      </c>
+      <c r="N78" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>294</v>
+      </c>
+      <c r="B79" t="n">
+        <v>88</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>sb</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>joint_belief</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>sb-at</t>
+        </is>
+      </c>
+      <c r="F79" t="n">
+        <v>4.666666666666667</v>
+      </c>
+      <c r="G79" t="n">
+        <v>4</v>
+      </c>
+      <c r="H79" t="n">
+        <v>3</v>
+      </c>
+      <c r="I79" t="n">
+        <v>6</v>
+      </c>
+      <c r="J79" t="n">
+        <v>3</v>
+      </c>
+      <c r="K79" t="n">
+        <v>2</v>
+      </c>
+      <c r="L79" t="n">
+        <v>0</v>
+      </c>
+      <c r="M79" t="n">
+        <v>1</v>
+      </c>
+      <c r="N79" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>295</v>
+      </c>
+      <c r="B80" t="n">
+        <v>87</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>common_belief</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>at-sb</t>
+        </is>
+      </c>
+      <c r="F80" t="n">
+        <v>4</v>
+      </c>
+      <c r="G80" t="n">
+        <v>4</v>
+      </c>
+      <c r="H80" t="n">
+        <v>3.666666666666667</v>
+      </c>
+      <c r="I80" t="n">
+        <v>6</v>
+      </c>
+      <c r="J80" t="n">
+        <v>1</v>
+      </c>
+      <c r="K80" t="n">
+        <v>0</v>
+      </c>
+      <c r="L80" t="n">
+        <v>1</v>
+      </c>
+      <c r="M80" t="n">
+        <v>0</v>
+      </c>
+      <c r="N80" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>295</v>
+      </c>
+      <c r="B81" t="n">
+        <v>87</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>sb</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>common_belief</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>at-sb</t>
+        </is>
+      </c>
+      <c r="F81" t="n">
+        <v>4</v>
+      </c>
+      <c r="G81" t="n">
+        <v>4</v>
+      </c>
+      <c r="H81" t="n">
+        <v>4</v>
+      </c>
+      <c r="I81" t="n">
+        <v>6</v>
+      </c>
+      <c r="J81" t="n">
+        <v>3</v>
+      </c>
+      <c r="K81" t="n">
+        <v>1</v>
+      </c>
+      <c r="L81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M81" t="n">
+        <v>1</v>
+      </c>
+      <c r="N81" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>296</v>
+      </c>
+      <c r="B82" t="n">
+        <v>88</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>joint_belief</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>sb-at</t>
+        </is>
+      </c>
+      <c r="F82" t="n">
+        <v>4.666666666666667</v>
+      </c>
+      <c r="G82" t="n">
+        <v>5</v>
+      </c>
+      <c r="H82" t="n">
+        <v>1</v>
+      </c>
+      <c r="I82" t="n">
+        <v>6</v>
+      </c>
+      <c r="J82" t="n">
+        <v>5</v>
+      </c>
+      <c r="K82" t="n">
+        <v>2</v>
+      </c>
+      <c r="L82" t="n">
+        <v>1</v>
+      </c>
+      <c r="M82" t="n">
+        <v>2</v>
+      </c>
+      <c r="N82" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>296</v>
+      </c>
+      <c r="B83" t="n">
+        <v>88</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>sb</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>joint_belief</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>sb-at</t>
+        </is>
+      </c>
+      <c r="F83" t="n">
+        <v>4.666666666666667</v>
+      </c>
+      <c r="G83" t="n">
+        <v>5</v>
+      </c>
+      <c r="H83" t="n">
+        <v>2</v>
+      </c>
+      <c r="I83" t="n">
+        <v>6</v>
+      </c>
+      <c r="J83" t="n">
+        <v>4</v>
+      </c>
+      <c r="K83" t="n">
+        <v>2</v>
+      </c>
+      <c r="L83" t="n">
+        <v>1</v>
+      </c>
+      <c r="M83" t="n">
+        <v>1</v>
+      </c>
+      <c r="N83" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>299</v>
+      </c>
+      <c r="B84" t="n">
+        <v>89</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>individual_belief_low</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>at-sb</t>
+        </is>
+      </c>
+      <c r="F84" t="n">
+        <v>4</v>
+      </c>
+      <c r="G84" t="n">
+        <v>3</v>
+      </c>
+      <c r="H84" t="n">
+        <v>2.666666666666667</v>
+      </c>
+      <c r="I84" t="n">
+        <v>6</v>
+      </c>
+      <c r="J84" t="n">
+        <v>5</v>
+      </c>
+      <c r="K84" t="n">
+        <v>2</v>
+      </c>
+      <c r="L84" t="n">
+        <v>2</v>
+      </c>
+      <c r="M84" t="n">
+        <v>1</v>
+      </c>
+      <c r="N84" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>299</v>
+      </c>
+      <c r="B85" t="n">
+        <v>89</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>sb</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>individual_belief_low</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>at-sb</t>
+        </is>
+      </c>
+      <c r="F85" t="n">
+        <v>4</v>
+      </c>
+      <c r="G85" t="n">
+        <v>3</v>
+      </c>
+      <c r="H85" t="n">
+        <v>3</v>
+      </c>
+      <c r="I85" t="n">
+        <v>6</v>
+      </c>
+      <c r="J85" t="n">
+        <v>2</v>
+      </c>
+      <c r="K85" t="n">
+        <v>2</v>
+      </c>
+      <c r="L85" t="n">
+        <v>0</v>
+      </c>
+      <c r="M85" t="n">
+        <v>0</v>
+      </c>
+      <c r="N85" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>300</v>
+      </c>
+      <c r="B86" t="n">
+        <v>88</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>joint_belief</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>sb-at</t>
+        </is>
+      </c>
+      <c r="F86" t="n">
+        <v>3.666666666666667</v>
+      </c>
+      <c r="G86" t="n">
+        <v>4</v>
+      </c>
+      <c r="H86" t="n">
+        <v>2</v>
+      </c>
+      <c r="I86" t="n">
+        <v>6</v>
+      </c>
+      <c r="J86" t="n">
+        <v>5</v>
+      </c>
+      <c r="K86" t="n">
+        <v>2</v>
+      </c>
+      <c r="L86" t="n">
+        <v>1</v>
+      </c>
+      <c r="M86" t="n">
+        <v>2</v>
+      </c>
+      <c r="N86" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>300</v>
+      </c>
+      <c r="B87" t="n">
+        <v>88</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>sb</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>joint_belief</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>sb-at</t>
+        </is>
+      </c>
+      <c r="F87" t="n">
+        <v>3.666666666666667</v>
+      </c>
+      <c r="G87" t="n">
+        <v>3</v>
+      </c>
+      <c r="H87" t="n">
+        <v>3.666666666666667</v>
+      </c>
+      <c r="I87" t="n">
+        <v>6</v>
+      </c>
+      <c r="J87" t="n">
+        <v>3</v>
+      </c>
+      <c r="K87" t="n">
+        <v>2</v>
+      </c>
+      <c r="L87" t="n">
+        <v>1</v>
+      </c>
+      <c r="M87" t="n">
+        <v>0</v>
+      </c>
+      <c r="N87" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>301</v>
+      </c>
+      <c r="B88" t="n">
+        <v>89</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>individual_belief_low</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>at-sb</t>
+        </is>
+      </c>
+      <c r="F88" t="n">
+        <v>4.333333333333333</v>
+      </c>
+      <c r="G88" t="n">
+        <v>3</v>
+      </c>
+      <c r="H88" t="n">
+        <v>4.333333333333333</v>
+      </c>
+      <c r="I88" t="n">
+        <v>6</v>
+      </c>
+      <c r="J88" t="n">
+        <v>4</v>
+      </c>
+      <c r="K88" t="n">
+        <v>2</v>
+      </c>
+      <c r="L88" t="n">
+        <v>2</v>
+      </c>
+      <c r="M88" t="n">
+        <v>0</v>
+      </c>
+      <c r="N88" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>301</v>
+      </c>
+      <c r="B89" t="n">
+        <v>89</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>sb</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>individual_belief_low</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>at-sb</t>
+        </is>
+      </c>
+      <c r="F89" t="n">
+        <v>4.333333333333333</v>
+      </c>
+      <c r="G89" t="n">
+        <v>2</v>
+      </c>
+      <c r="H89" t="n">
+        <v>4.666666666666667</v>
+      </c>
+      <c r="I89" t="n">
+        <v>6</v>
+      </c>
+      <c r="J89" t="n">
+        <v>2</v>
+      </c>
+      <c r="K89" t="n">
+        <v>1</v>
+      </c>
+      <c r="L89" t="n">
+        <v>0</v>
+      </c>
+      <c r="M89" t="n">
+        <v>1</v>
+      </c>
+      <c r="N89" t="n">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>